<commit_message>
Added Latest Export of Excel
</commit_message>
<xml_diff>
--- a/03_Learning_Management/00_Excel_Export/links.xlsx
+++ b/03_Learning_Management/00_Excel_Export/links.xlsx
@@ -421,10 +421,10 @@
         <v>System Design</v>
       </c>
       <c r="C2" t="str">
-        <v>Scalability,Load Balancing,Distributing traffic across servers</v>
+        <v>Networking,Proxy vs Reverse Proxy,Client-side vs server-side proxying</v>
       </c>
       <c r="D2" t="str">
-        <v>https://lnkd.in/ewTeu-58</v>
+        <v>https://lnkd.in/enEy9QYD</v>
       </c>
     </row>
     <row r="3">
@@ -435,10 +435,10 @@
         <v>System Design</v>
       </c>
       <c r="C3" t="str">
-        <v>Networking,Proxy vs Reverse Proxy,Client-side vs server-side proxying</v>
+        <v>Scaling</v>
       </c>
       <c r="D3" t="str">
-        <v>https://lnkd.in/enEy9QYD</v>
+        <v>https://lnkd.in/e8Gyr4G2 ( Go to 2:25:15 )</v>
       </c>
     </row>
     <row r="4">
@@ -449,10 +449,10 @@
         <v>System Design</v>
       </c>
       <c r="C4" t="str">
-        <v>Distributed Systems,CAP Theorem,Consistency vs Availability vs Partition Tolerance</v>
+        <v>Caching</v>
       </c>
       <c r="D4" t="str">
-        <v>https://lnkd.in/eePkq2kJ</v>
+        <v>https://lnkd.in/e8Gyr4G2 (Go to 1:39:08 )</v>
       </c>
     </row>
     <row r="5">
@@ -463,10 +463,10 @@
         <v>System Design</v>
       </c>
       <c r="C5" t="str">
-        <v>Database Scaling,Sharding,Horizontal partitioning of data</v>
+        <v>Sharding</v>
       </c>
       <c r="D5" t="str">
-        <v>https://lnkd.in/e8Gyr4G2</v>
+        <v>https://lnkd.in/e8Gyr4G2 (From 0:30 to 1:23:40)</v>
       </c>
     </row>
     <row r="6">
@@ -477,10 +477,10 @@
         <v>System Design</v>
       </c>
       <c r="C6" t="str">
-        <v>Reliability,Availability,System uptime and fault tolerance</v>
+        <v>Data Processing,Batch vs Stream Processing,Offline vs real-time processing</v>
       </c>
       <c r="D6" t="str">
-        <v>https://lnkd.in/eEQ5MAnC</v>
+        <v>https://lnkd.in/ez5v_suJ</v>
       </c>
     </row>
     <row r="7">
@@ -491,10 +491,10 @@
         <v>System Design</v>
       </c>
       <c r="C7" t="str">
-        <v>System Design,Services,Microservices vs Monolith</v>
+        <v>Architecture,Stateful vs Stateless,System design patterns</v>
       </c>
       <c r="D7" t="str">
-        <v>https://lnkd.in/exyDGmSe</v>
+        <v>https://lnkd.in/egXhAmY4</v>
       </c>
     </row>
     <row r="8">
@@ -505,10 +505,10 @@
         <v>System Design</v>
       </c>
       <c r="C8" t="str">
-        <v>Database,Databases in System Design,Choosing DB types and usage</v>
+        <v>Realtime Systems,Long Polling vs WebSockets,Realtime communication methods</v>
       </c>
       <c r="D8" t="str">
-        <v>https://lnkd.in/eifbKsr6</v>
+        <v>https://lnkd.in/eYZnk-93</v>
       </c>
     </row>
     <row r="9">
@@ -519,10 +519,10 @@
         <v>System Design</v>
       </c>
       <c r="C9" t="str">
-        <v>Database,Data Sharding &amp; Partitioning,Splitting large datasets</v>
+        <v>Concurrency,Concurrency vs Parallelism,Execution models</v>
       </c>
       <c r="D9" t="str">
-        <v>https://lnkd.in/eVhzCnW5</v>
+        <v>https://lnkd.in/eRpCq8KQ</v>
       </c>
     </row>
     <row r="10">
@@ -533,10 +533,10 @@
         <v>System Design</v>
       </c>
       <c r="C10" t="str">
-        <v>Distributed Systems,Algorithms,Consensus &amp; coordination algorithms</v>
+        <v>Data Structures,Bloom Filters,Probabilistic data structures</v>
       </c>
       <c r="D10" t="str">
-        <v>https://lnkd.in/eXiJ9_GV</v>
+        <v>https://lnkd.in/eq6hN3Nn</v>
       </c>
     </row>
     <row r="11">
@@ -547,10 +547,10 @@
         <v>System Design</v>
       </c>
       <c r="C11" t="str">
-        <v>Distributed Systems,Consistent Hashing,Load distribution technique</v>
+        <v>Distributed Systems,Message Queues,Async communication (Kafka, RabbitMQ)</v>
       </c>
       <c r="D11" t="str">
-        <v>https://lnkd.in/eYgXNHz4</v>
+        <v>https://lnkd.in/eKQWVxqw</v>
       </c>
     </row>
     <row r="12">
@@ -561,10 +561,10 @@
         <v>System Design</v>
       </c>
       <c r="C12" t="str">
-        <v>Data Engineering,CDC (Change Data Capture),Tracking data changes</v>
+        <v>Security,Rate Limiting,Throttling API requests</v>
       </c>
       <c r="D12" t="str">
-        <v>https://lnkd.in/efeP3fXP</v>
+        <v>https://lnkd.in/etby2w5C</v>
       </c>
     </row>
     <row r="13">
@@ -575,10 +575,10 @@
         <v>System Design</v>
       </c>
       <c r="C13" t="str">
-        <v>Caching,Caching Advanced,Advanced caching concepts</v>
+        <v>Performance,CDN,Content delivery optimization</v>
       </c>
       <c r="D13" t="str">
-        <v>https://lnkd.in/eqDfvdvB</v>
+        <v>https://lnkd.in/eCSccEkz</v>
       </c>
     </row>
     <row r="14">
@@ -589,10 +589,10 @@
         <v>System Design</v>
       </c>
       <c r="C14" t="str">
-        <v>Caching,Caching Strategies,Write-through, write-back, cache-aside</v>
+        <v>Caching,Cache Eviction Policies,LRU, LFU, FIFO</v>
       </c>
       <c r="D14" t="str">
-        <v>https://lnkd.in/eqFTdS_v</v>
+        <v>https://lnkd.in/ewB5MZ7z</v>
       </c>
     </row>
     <row r="15">
@@ -603,10 +603,10 @@
         <v>System Design</v>
       </c>
       <c r="C15" t="str">
-        <v>Caching,Cache Eviction Policies,LRU, LFU, FIFO</v>
+        <v>Caching,Caching Advanced,Advanced caching concepts</v>
       </c>
       <c r="D15" t="str">
-        <v>https://lnkd.in/ewB5MZ7z</v>
+        <v>https://lnkd.in/eqDfvdvB</v>
       </c>
     </row>
     <row r="16">
@@ -617,10 +617,10 @@
         <v>System Design</v>
       </c>
       <c r="C16" t="str">
-        <v>Performance,CDN,Content delivery optimization</v>
+        <v>Scalability,Load Balancing,Distributing traffic across servers</v>
       </c>
       <c r="D16" t="str">
-        <v>https://lnkd.in/eCSccEkz</v>
+        <v>https://lnkd.in/ewTeu-58</v>
       </c>
     </row>
     <row r="17">
@@ -631,10 +631,10 @@
         <v>System Design</v>
       </c>
       <c r="C17" t="str">
-        <v>Security,Rate Limiting,Throttling API requests</v>
+        <v>Distributed Systems,CAP Theorem,Consistency vs Availability vs Partition Tolerance</v>
       </c>
       <c r="D17" t="str">
-        <v>https://lnkd.in/etby2w5C</v>
+        <v>https://lnkd.in/eePkq2kJ</v>
       </c>
     </row>
     <row r="18">
@@ -645,10 +645,10 @@
         <v>System Design</v>
       </c>
       <c r="C18" t="str">
-        <v>Distributed Systems,Message Queues,Async communication (Kafka, RabbitMQ)</v>
+        <v>Database Scaling,Sharding,Horizontal partitioning of data</v>
       </c>
       <c r="D18" t="str">
-        <v>https://lnkd.in/eKQWVxqw</v>
+        <v>https://lnkd.in/e8Gyr4G2</v>
       </c>
     </row>
     <row r="19">
@@ -659,10 +659,10 @@
         <v>System Design</v>
       </c>
       <c r="C19" t="str">
-        <v>Data Structures,Bloom Filters,Probabilistic data structures</v>
+        <v>Reliability,Availability,System uptime and fault tolerance</v>
       </c>
       <c r="D19" t="str">
-        <v>https://lnkd.in/eq6hN3Nn</v>
+        <v>https://lnkd.in/eEQ5MAnC</v>
       </c>
     </row>
     <row r="20">
@@ -673,10 +673,10 @@
         <v>System Design</v>
       </c>
       <c r="C20" t="str">
-        <v>Concurrency,Concurrency vs Parallelism,Execution models</v>
+        <v>System Design,Services,Microservices vs Monolith</v>
       </c>
       <c r="D20" t="str">
-        <v>https://lnkd.in/eRpCq8KQ</v>
+        <v>https://lnkd.in/exyDGmSe</v>
       </c>
     </row>
     <row r="21">
@@ -687,10 +687,10 @@
         <v>System Design</v>
       </c>
       <c r="C21" t="str">
-        <v>Realtime Systems,Long Polling vs WebSockets,Realtime communication methods</v>
+        <v>Database,Data Sharding &amp; Partitioning,Splitting large datasets</v>
       </c>
       <c r="D21" t="str">
-        <v>https://lnkd.in/eYZnk-93</v>
+        <v>https://lnkd.in/eVhzCnW5</v>
       </c>
     </row>
     <row r="22">
@@ -701,10 +701,10 @@
         <v>System Design</v>
       </c>
       <c r="C22" t="str">
-        <v>Architecture,Stateful vs Stateless,System design patterns</v>
+        <v>Distributed Systems,Algorithms,Consensus &amp; coordination algorithms</v>
       </c>
       <c r="D22" t="str">
-        <v>https://lnkd.in/egXhAmY4</v>
+        <v>https://lnkd.in/eXiJ9_GV</v>
       </c>
     </row>
     <row r="23">
@@ -715,10 +715,10 @@
         <v>System Design</v>
       </c>
       <c r="C23" t="str">
-        <v>Data Processing,Batch vs Stream Processing,Offline vs real-time processing</v>
+        <v>Distributed Systems,Consistent Hashing,Load distribution technique</v>
       </c>
       <c r="D23" t="str">
-        <v>https://lnkd.in/ez5v_suJ</v>
+        <v>https://lnkd.in/eYgXNHz4</v>
       </c>
     </row>
     <row r="24">
@@ -729,10 +729,10 @@
         <v>System Design</v>
       </c>
       <c r="C24" t="str">
-        <v>Sharding</v>
+        <v>Data Engineering,CDC (Change Data Capture),Tracking data changes</v>
       </c>
       <c r="D24" t="str">
-        <v>https://lnkd.in/e8Gyr4G2 (From 0:30 to 1:23:40)</v>
+        <v>https://lnkd.in/efeP3fXP</v>
       </c>
     </row>
     <row r="25">
@@ -743,10 +743,10 @@
         <v>System Design</v>
       </c>
       <c r="C25" t="str">
-        <v>Caching</v>
+        <v>Caching,Caching Strategies,Write-through, write-back, cache-aside</v>
       </c>
       <c r="D25" t="str">
-        <v>https://lnkd.in/e8Gyr4G2 (Go to 1:39:08 )</v>
+        <v>https://lnkd.in/eqFTdS_v</v>
       </c>
     </row>
     <row r="26">
@@ -757,10 +757,10 @@
         <v>System Design</v>
       </c>
       <c r="C26" t="str">
-        <v>Scaling</v>
+        <v>Database,Databases in System Design,Choosing DB types and usage</v>
       </c>
       <c r="D26" t="str">
-        <v>https://lnkd.in/e8Gyr4G2 ( Go to 2:25:15 )</v>
+        <v>https://lnkd.in/eifbKsr6</v>
       </c>
     </row>
     <row r="27">
@@ -771,10 +771,10 @@
         <v>Backend</v>
       </c>
       <c r="C27" t="str">
-        <v>API Design,APIs,Basics of API design and usage</v>
+        <v>tRPC, gRPC, GraphQL, or REST</v>
       </c>
       <c r="D27" t="str">
-        <v>https://lnkd.in/ezwnCGqS</v>
+        <v>when to use what?</v>
       </c>
     </row>
     <row r="28">
@@ -785,10 +785,10 @@
         <v>Backend</v>
       </c>
       <c r="C28" t="str">
-        <v>API Design,API Gateways,Routing, authentication, aggregation</v>
+        <v>API Design,Idempotency,Safe retries in APIs</v>
       </c>
       <c r="D28" t="str">
-        <v>https://lnkd.in/eqNrc77q</v>
+        <v>https://lnkd.in/e-sB7a3w</v>
       </c>
     </row>
     <row r="29">
@@ -799,10 +799,10 @@
         <v>Backend</v>
       </c>
       <c r="C29" t="str">
-        <v>Security,JWT,Authentication using tokens</v>
+        <v>API Design,REST,RESTful principles</v>
       </c>
       <c r="D29" t="str">
-        <v>https://lnkd.in/eAnfnzm7</v>
+        <v>https://lnkd.in/eY2ACHFC</v>
       </c>
     </row>
     <row r="30">
@@ -813,10 +813,10 @@
         <v>Backend</v>
       </c>
       <c r="C30" t="str">
-        <v>API Communication,Webhooks,Event-driven HTTP callbacks</v>
+        <v>Concurrency,Sync vs Async,Synchronous vs asynchronous processing</v>
       </c>
       <c r="D30" t="str">
-        <v>https://lnkd.in/eF6gPzVJ</v>
+        <v>https://lnkd.in/ekrADFHy</v>
       </c>
     </row>
     <row r="31">
@@ -841,10 +841,10 @@
         <v>Backend</v>
       </c>
       <c r="C32" t="str">
-        <v>Concurrency,Sync vs Async,Synchronous vs asynchronous processing</v>
+        <v>API Communication,Webhooks,Event-driven HTTP callbacks</v>
       </c>
       <c r="D32" t="str">
-        <v>https://lnkd.in/ekrADFHy</v>
+        <v>https://lnkd.in/eF6gPzVJ</v>
       </c>
     </row>
     <row r="33">
@@ -855,10 +855,10 @@
         <v>Backend</v>
       </c>
       <c r="C33" t="str">
-        <v>API Design,REST,RESTful principles</v>
+        <v>Security,JWT,Authentication using tokens</v>
       </c>
       <c r="D33" t="str">
-        <v>https://lnkd.in/eY2ACHFC</v>
+        <v>https://lnkd.in/eAnfnzm7</v>
       </c>
     </row>
     <row r="34">
@@ -869,10 +869,10 @@
         <v>Backend</v>
       </c>
       <c r="C34" t="str">
-        <v>API Design,Idempotency,Safe retries in APIs</v>
+        <v>API Design,API Gateways,Routing, authentication, aggregation</v>
       </c>
       <c r="D34" t="str">
-        <v>https://lnkd.in/e-sB7a3w</v>
+        <v>https://lnkd.in/eqNrc77q</v>
       </c>
     </row>
     <row r="35">
@@ -883,10 +883,10 @@
         <v>Backend</v>
       </c>
       <c r="C35" t="str">
-        <v>tRPC, gRPC, GraphQL, or REST</v>
+        <v>API Design,APIs,Basics of API design and usage</v>
       </c>
       <c r="D35" t="str">
-        <v>when to use what?</v>
+        <v>https://lnkd.in/ezwnCGqS</v>
       </c>
     </row>
     <row r="36">

</xml_diff>

<commit_message>
Added Latest Export of Excel Sheets
</commit_message>
<xml_diff>
--- a/03_Learning_Management/00_Excel_Export/links.xlsx
+++ b/03_Learning_Management/00_Excel_Export/links.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -617,10 +617,10 @@
         <v>System Design</v>
       </c>
       <c r="C16" t="str">
-        <v>Scalability,Load Balancing,Distributing traffic across servers</v>
+        <v>Caching,Caching Strategies,Write-through, write-back, cache-aside</v>
       </c>
       <c r="D16" t="str">
-        <v>https://lnkd.in/ewTeu-58</v>
+        <v>https://lnkd.in/eqFTdS_v</v>
       </c>
     </row>
     <row r="17">
@@ -631,10 +631,10 @@
         <v>System Design</v>
       </c>
       <c r="C17" t="str">
-        <v>Distributed Systems,CAP Theorem,Consistency vs Availability vs Partition Tolerance</v>
+        <v>Scalability,Load Balancing,Distributing traffic across servers</v>
       </c>
       <c r="D17" t="str">
-        <v>https://lnkd.in/eePkq2kJ</v>
+        <v>https://lnkd.in/ewTeu-58</v>
       </c>
     </row>
     <row r="18">
@@ -645,10 +645,10 @@
         <v>System Design</v>
       </c>
       <c r="C18" t="str">
-        <v>Database Scaling,Sharding,Horizontal partitioning of data</v>
+        <v>Distributed Systems,CAP Theorem,Consistency vs Availability vs Partition Tolerance</v>
       </c>
       <c r="D18" t="str">
-        <v>https://lnkd.in/e8Gyr4G2</v>
+        <v>https://lnkd.in/eePkq2kJ</v>
       </c>
     </row>
     <row r="19">
@@ -659,10 +659,10 @@
         <v>System Design</v>
       </c>
       <c r="C19" t="str">
-        <v>Reliability,Availability,System uptime and fault tolerance</v>
+        <v>Database Scaling,Sharding,Horizontal partitioning of data</v>
       </c>
       <c r="D19" t="str">
-        <v>https://lnkd.in/eEQ5MAnC</v>
+        <v>https://lnkd.in/e8Gyr4G2</v>
       </c>
     </row>
     <row r="20">
@@ -673,10 +673,10 @@
         <v>System Design</v>
       </c>
       <c r="C20" t="str">
-        <v>System Design,Services,Microservices vs Monolith</v>
+        <v>Reliability,Availability,System uptime and fault tolerance</v>
       </c>
       <c r="D20" t="str">
-        <v>https://lnkd.in/exyDGmSe</v>
+        <v>https://lnkd.in/eEQ5MAnC</v>
       </c>
     </row>
     <row r="21">
@@ -687,10 +687,10 @@
         <v>System Design</v>
       </c>
       <c r="C21" t="str">
-        <v>Database,Data Sharding &amp; Partitioning,Splitting large datasets</v>
+        <v>System Design,Services,Microservices vs Monolith</v>
       </c>
       <c r="D21" t="str">
-        <v>https://lnkd.in/eVhzCnW5</v>
+        <v>https://lnkd.in/exyDGmSe</v>
       </c>
     </row>
     <row r="22">
@@ -701,10 +701,10 @@
         <v>System Design</v>
       </c>
       <c r="C22" t="str">
-        <v>Distributed Systems,Algorithms,Consensus &amp; coordination algorithms</v>
+        <v>Database,Databases in System Design,Choosing DB types and usage</v>
       </c>
       <c r="D22" t="str">
-        <v>https://lnkd.in/eXiJ9_GV</v>
+        <v>https://lnkd.in/eifbKsr6</v>
       </c>
     </row>
     <row r="23">
@@ -715,10 +715,10 @@
         <v>System Design</v>
       </c>
       <c r="C23" t="str">
-        <v>Distributed Systems,Consistent Hashing,Load distribution technique</v>
+        <v>Database,Data Sharding &amp; Partitioning,Splitting large datasets</v>
       </c>
       <c r="D23" t="str">
-        <v>https://lnkd.in/eYgXNHz4</v>
+        <v>https://lnkd.in/eVhzCnW5</v>
       </c>
     </row>
     <row r="24">
@@ -729,10 +729,10 @@
         <v>System Design</v>
       </c>
       <c r="C24" t="str">
-        <v>Data Engineering,CDC (Change Data Capture),Tracking data changes</v>
+        <v>Distributed Systems,Algorithms,Consensus &amp; coordination algorithms</v>
       </c>
       <c r="D24" t="str">
-        <v>https://lnkd.in/efeP3fXP</v>
+        <v>https://lnkd.in/eXiJ9_GV</v>
       </c>
     </row>
     <row r="25">
@@ -743,10 +743,10 @@
         <v>System Design</v>
       </c>
       <c r="C25" t="str">
-        <v>Caching,Caching Strategies,Write-through, write-back, cache-aside</v>
+        <v>Distributed Systems,Consistent Hashing,Load distribution technique</v>
       </c>
       <c r="D25" t="str">
-        <v>https://lnkd.in/eqFTdS_v</v>
+        <v>https://lnkd.in/eYgXNHz4</v>
       </c>
     </row>
     <row r="26">
@@ -757,10 +757,10 @@
         <v>System Design</v>
       </c>
       <c r="C26" t="str">
-        <v>Database,Databases in System Design,Choosing DB types and usage</v>
+        <v>Data Engineering,CDC (Change Data Capture),Tracking data changes</v>
       </c>
       <c r="D26" t="str">
-        <v>https://lnkd.in/eifbKsr6</v>
+        <v>https://lnkd.in/efeP3fXP</v>
       </c>
     </row>
     <row r="27">
@@ -771,10 +771,10 @@
         <v>Backend</v>
       </c>
       <c r="C27" t="str">
-        <v>tRPC, gRPC, GraphQL, or REST</v>
+        <v>API Design,APIs,Basics of API design and usage</v>
       </c>
       <c r="D27" t="str">
-        <v>when to use what?</v>
+        <v>https://lnkd.in/ezwnCGqS</v>
       </c>
     </row>
     <row r="28">
@@ -785,10 +785,10 @@
         <v>Backend</v>
       </c>
       <c r="C28" t="str">
-        <v>API Design,Idempotency,Safe retries in APIs</v>
+        <v>tRPC, gRPC, GraphQL, or REST</v>
       </c>
       <c r="D28" t="str">
-        <v>https://lnkd.in/e-sB7a3w</v>
+        <v>when to use what?</v>
       </c>
     </row>
     <row r="29">
@@ -799,10 +799,10 @@
         <v>Backend</v>
       </c>
       <c r="C29" t="str">
-        <v>API Design,REST,RESTful principles</v>
+        <v>API Design,Idempotency,Safe retries in APIs</v>
       </c>
       <c r="D29" t="str">
-        <v>https://lnkd.in/eY2ACHFC</v>
+        <v>https://lnkd.in/e-sB7a3w</v>
       </c>
     </row>
     <row r="30">
@@ -813,10 +813,10 @@
         <v>Backend</v>
       </c>
       <c r="C30" t="str">
-        <v>Concurrency,Sync vs Async,Synchronous vs asynchronous processing</v>
+        <v>API Design,REST,RESTful principles</v>
       </c>
       <c r="D30" t="str">
-        <v>https://lnkd.in/ekrADFHy</v>
+        <v>https://lnkd.in/eY2ACHFC</v>
       </c>
     </row>
     <row r="31">
@@ -827,10 +827,10 @@
         <v>Backend</v>
       </c>
       <c r="C31" t="str">
-        <v>API Architecture,API Paradigms,tRPC vs gRPC vs GraphQL vs REST</v>
+        <v>Concurrency,Sync vs Async,Synchronous vs asynchronous processing</v>
       </c>
       <c r="D31" t="str">
-        <v>https://lnkd.in/eydTuVj3</v>
+        <v>https://lnkd.in/ekrADFHy</v>
       </c>
     </row>
     <row r="32">
@@ -841,10 +841,10 @@
         <v>Backend</v>
       </c>
       <c r="C32" t="str">
-        <v>API Communication,Webhooks,Event-driven HTTP callbacks</v>
+        <v>API Architecture,API Paradigms,tRPC vs gRPC vs GraphQL vs REST</v>
       </c>
       <c r="D32" t="str">
-        <v>https://lnkd.in/eF6gPzVJ</v>
+        <v>https://lnkd.in/eydTuVj3</v>
       </c>
     </row>
     <row r="33">
@@ -855,10 +855,10 @@
         <v>Backend</v>
       </c>
       <c r="C33" t="str">
-        <v>Security,JWT,Authentication using tokens</v>
+        <v>API Communication,Webhooks,Event-driven HTTP callbacks</v>
       </c>
       <c r="D33" t="str">
-        <v>https://lnkd.in/eAnfnzm7</v>
+        <v>https://lnkd.in/eF6gPzVJ</v>
       </c>
     </row>
     <row r="34">
@@ -869,10 +869,10 @@
         <v>Backend</v>
       </c>
       <c r="C34" t="str">
-        <v>API Design,API Gateways,Routing, authentication, aggregation</v>
+        <v>Security,JWT,Authentication using tokens</v>
       </c>
       <c r="D34" t="str">
-        <v>https://lnkd.in/eqNrc77q</v>
+        <v>https://lnkd.in/eAnfnzm7</v>
       </c>
     </row>
     <row r="35">
@@ -883,10 +883,10 @@
         <v>Backend</v>
       </c>
       <c r="C35" t="str">
-        <v>API Design,APIs,Basics of API design and usage</v>
+        <v>API Design,API Gateways,Routing, authentication, aggregation</v>
       </c>
       <c r="D35" t="str">
-        <v>https://lnkd.in/ezwnCGqS</v>
+        <v>https://lnkd.in/eqNrc77q</v>
       </c>
     </row>
     <row r="36">
@@ -894,13 +894,13 @@
         <v>WebDev</v>
       </c>
       <c r="B36" t="str">
-        <v>SQL</v>
+        <v>DSA</v>
       </c>
       <c r="C36" t="str">
-        <v>Database,SQL vs NoSQL,Relational vs non-relational DBs</v>
+        <v xml:space="preserve">Sharpener DSA Topics </v>
       </c>
       <c r="D36" t="str">
-        <v>https://lnkd.in/entah3zc</v>
+        <v>https://docs.google.com/spreadsheets/d/1OBl8_DEUH8-hJaMRlU0Gqee_XbsgX5CIFyPJyEgGEG0/edit?gid=0#gid=0</v>
       </c>
     </row>
     <row r="37">
@@ -911,15 +911,29 @@
         <v>SQL</v>
       </c>
       <c r="C37" t="str">
+        <v>Database,SQL vs NoSQL,Relational vs non-relational DBs</v>
+      </c>
+      <c r="D37" t="str">
+        <v>https://lnkd.in/entah3zc</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>WebDev</v>
+      </c>
+      <c r="B38" t="str">
+        <v>SQL</v>
+      </c>
+      <c r="C38" t="str">
         <v>Database,ACID Transactions,Reliability guarantees in DBs</v>
       </c>
-      <c r="D37" t="str">
+      <c r="D38" t="str">
         <v>https://lnkd.in/etXk_wa4</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D38"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>